<commit_message>
fix gap analysis naming
</commit_message>
<xml_diff>
--- a/final_artifact/gap-analysis.xlsx
+++ b/final_artifact/gap-analysis.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fariz/Downloads/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fariz/repositories/significancetestXNLP/final_artifact/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A790E72-75C2-9746-946E-4B48DC4FD183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{706BADD7-0EFA-4347-93EA-E0E2EC12F064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17140" xr2:uid="{A1799BBB-4479-DC43-BE44-E88E968B2414}"/>
   </bookViews>

</xml_diff>